<commit_message>
up clean code and new data
cleaning code to remove errors and add indicators
new data downloaded from the zonal app stat _ new grid
</commit_message>
<xml_diff>
--- a/Data/IND/FABLE.xlsx
+++ b/Data/IND/FABLE.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Clara DOUZAL\Documents\Github Desktop\DownscalingFABLE\Data\IND\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FB095AB-18A7-41FA-8FAD-1C5083F8677E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD7FB42B-4DEA-49DE-855B-4F741C3C9083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{10461ED0-0A96-44CE-86CA-319C52581F24}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="1" xr2:uid="{10461ED0-0A96-44CE-86CA-319C52581F24}"/>
   </bookViews>
   <sheets>
     <sheet name="CurrentTrends" sheetId="1" r:id="rId1"/>
-    <sheet name="NationalCommitments" sheetId="2" r:id="rId2"/>
-    <sheet name="GlobalSustainability" sheetId="3" r:id="rId3"/>
+    <sheet name="Baseline" sheetId="4" r:id="rId2"/>
+    <sheet name="NationalCommitments" sheetId="2" r:id="rId3"/>
+    <sheet name="GlobalSustainability" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="24">
   <si>
     <t>LandCoverInit</t>
   </si>
@@ -83,6 +84,33 @@
   </si>
   <si>
     <t>NewForest</t>
+  </si>
+  <si>
+    <t>LandCover</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>cropland</t>
+  </si>
+  <si>
+    <t>pasture</t>
+  </si>
+  <si>
+    <t>urban</t>
+  </si>
+  <si>
+    <t>newforest</t>
+  </si>
+  <si>
+    <t>forest</t>
+  </si>
+  <si>
+    <t>otherland</t>
+  </si>
+  <si>
+    <t>not relevant</t>
   </si>
 </sst>
 </file>
@@ -2273,6 +2301,80 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22657D6F-409E-453B-9A78-12BCC2059112}">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2">
+        <v>169413</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3">
+        <v>10262.754646368547</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4">
+        <v>2227.6714938742321</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6">
+        <v>67591</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7">
+        <v>47824.573859757249</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0090468E-82DD-4BA2-B54A-6FCCDCE9F12F}">
   <dimension ref="A1:I61"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -4051,7 +4153,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE7301B5-1FC0-446C-8B04-03B45EA22A45}">
   <dimension ref="A1:I61"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>

</xml_diff>